<commit_message>
WIP for specification reader step
</commit_message>
<xml_diff>
--- a/src/test.dataExchange/resources/filesToIngest/mfpDemo.xlsx
+++ b/src/test.dataExchange/resources/filesToIngest/mfpDemo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rachowdhury\Documents\Software\mtf-dm-automation-test-api\src\test.dataExchange\resources\filesToIngest\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43CBD866-25B2-44E5-BC59-E76D8EE24E32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36BE23CA-5E5E-4851-8244-4EF155EC55F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{19ED86A4-C2F1-4297-8EB6-669432289AF5}"/>
   </bookViews>
@@ -36,10 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="24">
-  <si>
-    <t>SAMPLE DATA</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="22">
   <si>
     <t>IPAY</t>
   </si>
@@ -83,10 +80,6 @@
     <t>Remarks</t>
   </si>
   <si>
-    <t xml:space="preserve">Notes
-- Additional Fields will be added so breakdown by Manu and/or Drug Level. If so, no need for crosswalk files. </t>
-  </si>
-  <si>
     <t>ELIQUIS</t>
   </si>
   <si>
@@ -118,7 +111,7 @@
   <numFmts count="1">
     <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
   </numFmts>
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="18">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -253,17 +246,8 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b/>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="35">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -446,12 +430,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -616,7 +594,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -628,9 +606,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1007,104 +982,119 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9669907-CFD9-41C9-BD8E-B33EA6BCF659}">
-  <dimension ref="A1:X143"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:X142"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
-    <col min="4" max="4" width="12.44140625" customWidth="1"/>
-    <col min="7" max="7" width="16.88671875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.3984375" customWidth="1"/>
+    <col min="7" max="7" width="16.8984375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.296875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.3984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A1" s="6" t="s">
+    <row r="1" spans="1:24" s="3" customFormat="1" ht="90.75" customHeight="1">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
-      <c r="F1" s="6"/>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6"/>
-      <c r="I1" s="6"/>
-      <c r="J1" s="6"/>
-      <c r="K1" s="6"/>
-      <c r="L1" s="6"/>
-      <c r="M1" s="6"/>
-      <c r="N1" s="6"/>
-      <c r="O1" s="6"/>
-      <c r="P1" s="6"/>
-      <c r="Q1" s="6"/>
-    </row>
-    <row r="2" spans="1:24" s="3" customFormat="1" ht="90.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="3" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="J1" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="K1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="K2" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="L2" s="3" t="s">
+      <c r="M1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="M2" s="3" t="s">
+      <c r="N1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="N2" s="3" t="s">
+      <c r="S1" s="5"/>
+      <c r="T1" s="5"/>
+      <c r="U1" s="5"/>
+      <c r="V1" s="5"/>
+      <c r="W1" s="5"/>
+      <c r="X1" s="5"/>
+    </row>
+    <row r="2" spans="1:24">
+      <c r="A2">
+        <v>2026</v>
+      </c>
+      <c r="B2" t="s">
         <v>14</v>
       </c>
-      <c r="S2" s="5" t="s">
+      <c r="C2" t="s">
         <v>15</v>
       </c>
-      <c r="T2" s="5"/>
-      <c r="U2" s="5"/>
-      <c r="V2" s="5"/>
-      <c r="W2" s="5"/>
-      <c r="X2" s="5"/>
-    </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="D2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G2" s="1">
+        <v>46023</v>
+      </c>
+      <c r="I2" s="2">
+        <v>231</v>
+      </c>
+      <c r="J2" s="2">
+        <v>4.1450719999999999</v>
+      </c>
+      <c r="K2" s="2">
+        <v>248.7</v>
+      </c>
+      <c r="L2" s="1">
+        <v>45519</v>
+      </c>
+      <c r="M2" t="s">
+        <v>18</v>
+      </c>
+      <c r="N2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:24">
       <c r="A3">
         <v>2026</v>
       </c>
       <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" t="s">
         <v>16</v>
       </c>
-      <c r="C3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D3" t="s">
-        <v>18</v>
-      </c>
       <c r="E3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G3" s="1">
         <v>46023</v>
@@ -1116,33 +1106,33 @@
         <v>4.1450719999999999</v>
       </c>
       <c r="K3" s="2">
-        <v>248.7</v>
+        <v>414.51</v>
       </c>
       <c r="L3" s="1">
         <v>45519</v>
       </c>
       <c r="M3" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="N3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:24">
       <c r="A4">
         <v>2026</v>
       </c>
       <c r="B4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" t="s">
         <v>16</v>
       </c>
-      <c r="C4" t="s">
-        <v>17</v>
-      </c>
-      <c r="D4" t="s">
-        <v>18</v>
-      </c>
       <c r="E4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G4" s="1">
         <v>46023</v>
@@ -1154,1026 +1144,987 @@
         <v>4.1450719999999999</v>
       </c>
       <c r="K4" s="2">
-        <v>414.51</v>
+        <v>746.11</v>
       </c>
       <c r="L4" s="1">
         <v>45519</v>
       </c>
       <c r="M4" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="N4" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A5">
-        <v>2026</v>
-      </c>
-      <c r="B5" t="s">
-        <v>16</v>
-      </c>
-      <c r="C5" t="s">
-        <v>17</v>
-      </c>
-      <c r="D5" t="s">
-        <v>18</v>
-      </c>
-      <c r="E5" t="s">
-        <v>23</v>
-      </c>
-      <c r="G5" s="1">
-        <v>46023</v>
-      </c>
-      <c r="I5" s="2">
-        <v>231</v>
-      </c>
-      <c r="J5" s="2">
-        <v>4.1450719999999999</v>
-      </c>
-      <c r="K5" s="2">
-        <v>746.11</v>
-      </c>
-      <c r="L5" s="1">
-        <v>45519</v>
-      </c>
-      <c r="M5" t="s">
-        <v>20</v>
-      </c>
-      <c r="N5" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:24">
+      <c r="G5" s="1"/>
+      <c r="I5" s="2"/>
+      <c r="J5" s="2"/>
+      <c r="K5" s="2"/>
+      <c r="L5" s="1"/>
+    </row>
+    <row r="6" spans="1:24">
       <c r="G6" s="1"/>
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
       <c r="K6" s="2"/>
       <c r="L6" s="1"/>
     </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:24">
       <c r="G7" s="1"/>
       <c r="I7" s="2"/>
       <c r="J7" s="2"/>
       <c r="K7" s="2"/>
       <c r="L7" s="1"/>
     </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:24">
       <c r="G8" s="1"/>
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
       <c r="K8" s="2"/>
       <c r="L8" s="1"/>
     </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:24">
       <c r="G9" s="1"/>
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
       <c r="K9" s="2"/>
       <c r="L9" s="1"/>
     </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:24">
       <c r="G10" s="1"/>
       <c r="I10" s="2"/>
       <c r="J10" s="2"/>
       <c r="K10" s="2"/>
       <c r="L10" s="1"/>
     </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:24">
       <c r="G11" s="1"/>
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
       <c r="K11" s="2"/>
       <c r="L11" s="1"/>
     </row>
-    <row r="12" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:24">
       <c r="G12" s="1"/>
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
       <c r="L12" s="1"/>
     </row>
-    <row r="13" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:24">
       <c r="G13" s="1"/>
       <c r="I13" s="2"/>
       <c r="J13" s="2"/>
       <c r="K13" s="2"/>
       <c r="L13" s="1"/>
     </row>
-    <row r="14" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:24">
       <c r="G14" s="1"/>
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>
       <c r="L14" s="1"/>
     </row>
-    <row r="15" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:24">
       <c r="G15" s="1"/>
       <c r="I15" s="2"/>
       <c r="J15" s="2"/>
       <c r="K15" s="2"/>
       <c r="L15" s="1"/>
     </row>
-    <row r="16" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:24">
       <c r="G16" s="1"/>
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
       <c r="K16" s="2"/>
       <c r="L16" s="1"/>
     </row>
-    <row r="17" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="17" spans="7:12">
       <c r="G17" s="1"/>
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
       <c r="K17" s="2"/>
       <c r="L17" s="1"/>
     </row>
-    <row r="18" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="18" spans="7:12">
       <c r="G18" s="1"/>
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
       <c r="K18" s="2"/>
       <c r="L18" s="1"/>
     </row>
-    <row r="19" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="19" spans="7:12">
       <c r="G19" s="1"/>
       <c r="I19" s="2"/>
       <c r="J19" s="2"/>
       <c r="K19" s="2"/>
       <c r="L19" s="1"/>
     </row>
-    <row r="20" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="20" spans="7:12">
       <c r="G20" s="1"/>
       <c r="I20" s="2"/>
       <c r="J20" s="2"/>
       <c r="K20" s="2"/>
       <c r="L20" s="1"/>
     </row>
-    <row r="21" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="21" spans="7:12">
       <c r="G21" s="1"/>
       <c r="I21" s="2"/>
       <c r="J21" s="2"/>
       <c r="K21" s="2"/>
       <c r="L21" s="1"/>
     </row>
-    <row r="22" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="22" spans="7:12">
       <c r="G22" s="1"/>
       <c r="I22" s="2"/>
       <c r="J22" s="2"/>
       <c r="K22" s="2"/>
       <c r="L22" s="1"/>
     </row>
-    <row r="23" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="23" spans="7:12">
       <c r="G23" s="1"/>
       <c r="I23" s="2"/>
       <c r="J23" s="2"/>
       <c r="K23" s="2"/>
       <c r="L23" s="1"/>
     </row>
-    <row r="24" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="24" spans="7:12">
       <c r="G24" s="1"/>
       <c r="I24" s="2"/>
       <c r="J24" s="2"/>
       <c r="K24" s="2"/>
       <c r="L24" s="1"/>
     </row>
-    <row r="25" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="25" spans="7:12">
       <c r="G25" s="1"/>
       <c r="I25" s="2"/>
       <c r="J25" s="2"/>
       <c r="K25" s="2"/>
       <c r="L25" s="1"/>
     </row>
-    <row r="26" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="26" spans="7:12">
       <c r="G26" s="1"/>
       <c r="I26" s="2"/>
       <c r="J26" s="2"/>
       <c r="K26" s="2"/>
       <c r="L26" s="1"/>
     </row>
-    <row r="27" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="27" spans="7:12">
       <c r="G27" s="1"/>
       <c r="I27" s="2"/>
       <c r="J27" s="2"/>
       <c r="K27" s="2"/>
       <c r="L27" s="1"/>
     </row>
-    <row r="28" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="28" spans="7:12">
       <c r="G28" s="1"/>
       <c r="I28" s="2"/>
       <c r="J28" s="2"/>
       <c r="K28" s="2"/>
       <c r="L28" s="1"/>
     </row>
-    <row r="29" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="29" spans="7:12">
       <c r="G29" s="1"/>
       <c r="I29" s="2"/>
       <c r="J29" s="2"/>
       <c r="K29" s="2"/>
       <c r="L29" s="1"/>
     </row>
-    <row r="30" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="30" spans="7:12">
       <c r="G30" s="1"/>
       <c r="I30" s="2"/>
       <c r="J30" s="2"/>
       <c r="K30" s="2"/>
       <c r="L30" s="1"/>
     </row>
-    <row r="31" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="31" spans="7:12">
       <c r="G31" s="1"/>
       <c r="I31" s="2"/>
       <c r="J31" s="2"/>
       <c r="K31" s="2"/>
       <c r="L31" s="1"/>
     </row>
-    <row r="32" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="32" spans="7:12">
       <c r="G32" s="1"/>
       <c r="I32" s="2"/>
       <c r="J32" s="2"/>
       <c r="K32" s="2"/>
       <c r="L32" s="1"/>
     </row>
-    <row r="33" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="33" spans="7:12">
       <c r="G33" s="1"/>
       <c r="I33" s="2"/>
       <c r="J33" s="2"/>
       <c r="K33" s="2"/>
       <c r="L33" s="1"/>
     </row>
-    <row r="34" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="34" spans="7:12">
       <c r="G34" s="1"/>
       <c r="I34" s="2"/>
       <c r="J34" s="2"/>
       <c r="K34" s="2"/>
       <c r="L34" s="1"/>
     </row>
-    <row r="35" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="35" spans="7:12">
       <c r="G35" s="1"/>
       <c r="I35" s="2"/>
       <c r="J35" s="2"/>
       <c r="K35" s="2"/>
       <c r="L35" s="1"/>
     </row>
-    <row r="36" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="36" spans="7:12">
       <c r="G36" s="1"/>
       <c r="I36" s="2"/>
       <c r="J36" s="2"/>
       <c r="K36" s="2"/>
       <c r="L36" s="1"/>
     </row>
-    <row r="37" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="37" spans="7:12">
       <c r="G37" s="1"/>
       <c r="I37" s="2"/>
       <c r="J37" s="2"/>
       <c r="K37" s="2"/>
       <c r="L37" s="1"/>
     </row>
-    <row r="38" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="38" spans="7:12">
       <c r="G38" s="1"/>
       <c r="I38" s="2"/>
       <c r="J38" s="2"/>
       <c r="K38" s="2"/>
       <c r="L38" s="1"/>
     </row>
-    <row r="39" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="39" spans="7:12">
       <c r="G39" s="1"/>
       <c r="I39" s="2"/>
       <c r="J39" s="2"/>
       <c r="K39" s="2"/>
       <c r="L39" s="1"/>
     </row>
-    <row r="40" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="40" spans="7:12">
       <c r="G40" s="1"/>
       <c r="I40" s="2"/>
       <c r="J40" s="2"/>
       <c r="K40" s="2"/>
       <c r="L40" s="1"/>
     </row>
-    <row r="41" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="41" spans="7:12">
       <c r="G41" s="1"/>
       <c r="I41" s="2"/>
       <c r="J41" s="2"/>
       <c r="K41" s="2"/>
       <c r="L41" s="1"/>
     </row>
-    <row r="42" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="42" spans="7:12">
       <c r="G42" s="1"/>
       <c r="I42" s="2"/>
       <c r="J42" s="2"/>
       <c r="K42" s="2"/>
       <c r="L42" s="1"/>
     </row>
-    <row r="43" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="43" spans="7:12">
       <c r="G43" s="1"/>
       <c r="I43" s="2"/>
       <c r="J43" s="2"/>
       <c r="K43" s="2"/>
       <c r="L43" s="1"/>
     </row>
-    <row r="44" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="44" spans="7:12">
       <c r="G44" s="1"/>
       <c r="I44" s="2"/>
       <c r="J44" s="2"/>
       <c r="K44" s="2"/>
       <c r="L44" s="1"/>
     </row>
-    <row r="45" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="45" spans="7:12">
       <c r="G45" s="1"/>
       <c r="I45" s="2"/>
       <c r="J45" s="2"/>
       <c r="K45" s="2"/>
       <c r="L45" s="1"/>
     </row>
-    <row r="46" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="46" spans="7:12">
       <c r="G46" s="1"/>
       <c r="I46" s="2"/>
       <c r="J46" s="2"/>
       <c r="K46" s="2"/>
       <c r="L46" s="1"/>
     </row>
-    <row r="47" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="47" spans="7:12">
       <c r="G47" s="1"/>
       <c r="I47" s="2"/>
       <c r="J47" s="2"/>
       <c r="K47" s="2"/>
       <c r="L47" s="1"/>
     </row>
-    <row r="48" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="48" spans="7:12">
       <c r="G48" s="1"/>
       <c r="I48" s="2"/>
       <c r="J48" s="2"/>
       <c r="K48" s="2"/>
       <c r="L48" s="1"/>
     </row>
-    <row r="49" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="49" spans="7:12">
       <c r="G49" s="1"/>
       <c r="I49" s="2"/>
       <c r="J49" s="2"/>
       <c r="K49" s="2"/>
       <c r="L49" s="1"/>
     </row>
-    <row r="50" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="50" spans="7:12">
       <c r="G50" s="1"/>
       <c r="I50" s="2"/>
       <c r="J50" s="2"/>
       <c r="K50" s="2"/>
       <c r="L50" s="1"/>
     </row>
-    <row r="51" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="51" spans="7:12">
       <c r="G51" s="1"/>
       <c r="I51" s="2"/>
       <c r="J51" s="2"/>
       <c r="K51" s="2"/>
       <c r="L51" s="1"/>
     </row>
-    <row r="52" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="52" spans="7:12">
       <c r="G52" s="1"/>
       <c r="I52" s="2"/>
       <c r="J52" s="2"/>
       <c r="K52" s="2"/>
       <c r="L52" s="1"/>
     </row>
-    <row r="53" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="53" spans="7:12">
       <c r="G53" s="1"/>
       <c r="I53" s="2"/>
       <c r="J53" s="2"/>
       <c r="K53" s="2"/>
       <c r="L53" s="1"/>
     </row>
-    <row r="54" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="54" spans="7:12">
       <c r="G54" s="1"/>
       <c r="I54" s="2"/>
       <c r="J54" s="2"/>
       <c r="K54" s="2"/>
       <c r="L54" s="1"/>
     </row>
-    <row r="55" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="55" spans="7:12">
       <c r="G55" s="1"/>
       <c r="I55" s="2"/>
       <c r="J55" s="2"/>
       <c r="K55" s="2"/>
       <c r="L55" s="1"/>
     </row>
-    <row r="56" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="56" spans="7:12">
       <c r="G56" s="1"/>
       <c r="I56" s="2"/>
       <c r="J56" s="2"/>
       <c r="K56" s="2"/>
       <c r="L56" s="1"/>
     </row>
-    <row r="57" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="57" spans="7:12">
       <c r="G57" s="1"/>
       <c r="I57" s="2"/>
       <c r="J57" s="2"/>
       <c r="K57" s="2"/>
       <c r="L57" s="1"/>
     </row>
-    <row r="58" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="58" spans="7:12">
       <c r="G58" s="1"/>
       <c r="I58" s="2"/>
       <c r="J58" s="2"/>
       <c r="K58" s="2"/>
       <c r="L58" s="1"/>
     </row>
-    <row r="59" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="59" spans="7:12">
       <c r="G59" s="1"/>
       <c r="I59" s="2"/>
       <c r="J59" s="2"/>
       <c r="K59" s="2"/>
       <c r="L59" s="1"/>
     </row>
-    <row r="60" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="60" spans="7:12">
       <c r="G60" s="1"/>
       <c r="I60" s="2"/>
       <c r="J60" s="2"/>
       <c r="K60" s="2"/>
       <c r="L60" s="1"/>
     </row>
-    <row r="61" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="61" spans="7:12">
       <c r="G61" s="1"/>
       <c r="I61" s="2"/>
       <c r="J61" s="2"/>
       <c r="K61" s="2"/>
       <c r="L61" s="1"/>
     </row>
-    <row r="62" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="62" spans="7:12">
       <c r="G62" s="1"/>
       <c r="I62" s="2"/>
       <c r="J62" s="2"/>
       <c r="K62" s="2"/>
       <c r="L62" s="1"/>
     </row>
-    <row r="63" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="63" spans="7:12">
       <c r="G63" s="1"/>
       <c r="I63" s="2"/>
       <c r="J63" s="2"/>
       <c r="K63" s="2"/>
       <c r="L63" s="1"/>
     </row>
-    <row r="64" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="64" spans="7:12">
       <c r="G64" s="1"/>
       <c r="I64" s="2"/>
       <c r="J64" s="2"/>
       <c r="K64" s="2"/>
       <c r="L64" s="1"/>
     </row>
-    <row r="65" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="65" spans="7:12">
       <c r="G65" s="1"/>
       <c r="I65" s="2"/>
       <c r="J65" s="2"/>
       <c r="K65" s="2"/>
       <c r="L65" s="1"/>
     </row>
-    <row r="66" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="66" spans="7:12">
       <c r="G66" s="1"/>
       <c r="I66" s="2"/>
       <c r="J66" s="2"/>
       <c r="K66" s="2"/>
       <c r="L66" s="1"/>
     </row>
-    <row r="67" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="67" spans="7:12">
       <c r="G67" s="1"/>
       <c r="I67" s="2"/>
       <c r="J67" s="2"/>
       <c r="K67" s="2"/>
       <c r="L67" s="1"/>
     </row>
-    <row r="68" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="68" spans="7:12">
       <c r="G68" s="1"/>
       <c r="I68" s="2"/>
       <c r="J68" s="2"/>
       <c r="K68" s="2"/>
       <c r="L68" s="1"/>
     </row>
-    <row r="69" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="69" spans="7:12">
       <c r="G69" s="1"/>
       <c r="I69" s="2"/>
       <c r="J69" s="2"/>
       <c r="K69" s="2"/>
       <c r="L69" s="1"/>
     </row>
-    <row r="70" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="70" spans="7:12">
       <c r="G70" s="1"/>
       <c r="I70" s="2"/>
       <c r="J70" s="2"/>
       <c r="K70" s="2"/>
       <c r="L70" s="1"/>
     </row>
-    <row r="71" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="71" spans="7:12">
       <c r="G71" s="1"/>
       <c r="I71" s="2"/>
       <c r="J71" s="2"/>
       <c r="K71" s="2"/>
       <c r="L71" s="1"/>
     </row>
-    <row r="72" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="72" spans="7:12">
       <c r="G72" s="1"/>
       <c r="I72" s="2"/>
       <c r="J72" s="2"/>
       <c r="K72" s="2"/>
       <c r="L72" s="1"/>
     </row>
-    <row r="73" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="73" spans="7:12">
       <c r="G73" s="1"/>
       <c r="I73" s="2"/>
       <c r="J73" s="2"/>
       <c r="K73" s="2"/>
       <c r="L73" s="1"/>
     </row>
-    <row r="74" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="74" spans="7:12">
       <c r="G74" s="1"/>
       <c r="I74" s="2"/>
       <c r="J74" s="2"/>
       <c r="K74" s="2"/>
       <c r="L74" s="1"/>
     </row>
-    <row r="75" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="75" spans="7:12">
       <c r="G75" s="1"/>
       <c r="I75" s="2"/>
       <c r="J75" s="2"/>
       <c r="K75" s="2"/>
       <c r="L75" s="1"/>
     </row>
-    <row r="76" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="76" spans="7:12">
       <c r="G76" s="1"/>
       <c r="I76" s="2"/>
       <c r="J76" s="2"/>
       <c r="K76" s="2"/>
       <c r="L76" s="1"/>
     </row>
-    <row r="77" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="77" spans="7:12">
       <c r="G77" s="1"/>
       <c r="I77" s="2"/>
       <c r="J77" s="2"/>
       <c r="K77" s="2"/>
       <c r="L77" s="1"/>
     </row>
-    <row r="78" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="78" spans="7:12">
       <c r="G78" s="1"/>
       <c r="I78" s="2"/>
       <c r="J78" s="2"/>
       <c r="K78" s="2"/>
       <c r="L78" s="1"/>
     </row>
-    <row r="79" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="79" spans="7:12">
       <c r="G79" s="1"/>
       <c r="I79" s="2"/>
       <c r="J79" s="2"/>
       <c r="K79" s="2"/>
       <c r="L79" s="1"/>
     </row>
-    <row r="80" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="80" spans="7:12">
       <c r="G80" s="1"/>
       <c r="I80" s="2"/>
       <c r="J80" s="2"/>
       <c r="K80" s="2"/>
       <c r="L80" s="1"/>
     </row>
-    <row r="81" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="81" spans="7:12">
       <c r="G81" s="1"/>
       <c r="I81" s="2"/>
       <c r="J81" s="2"/>
       <c r="K81" s="2"/>
       <c r="L81" s="1"/>
     </row>
-    <row r="82" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="82" spans="7:12">
       <c r="G82" s="1"/>
       <c r="I82" s="2"/>
       <c r="J82" s="2"/>
       <c r="K82" s="2"/>
       <c r="L82" s="1"/>
     </row>
-    <row r="83" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="83" spans="7:12">
       <c r="G83" s="1"/>
       <c r="I83" s="2"/>
       <c r="J83" s="2"/>
       <c r="K83" s="2"/>
       <c r="L83" s="1"/>
     </row>
-    <row r="84" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="84" spans="7:12">
       <c r="G84" s="1"/>
       <c r="I84" s="2"/>
       <c r="J84" s="2"/>
       <c r="K84" s="2"/>
       <c r="L84" s="1"/>
     </row>
-    <row r="85" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="85" spans="7:12">
       <c r="G85" s="1"/>
       <c r="I85" s="2"/>
       <c r="J85" s="2"/>
       <c r="K85" s="2"/>
       <c r="L85" s="1"/>
     </row>
-    <row r="86" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="86" spans="7:12">
       <c r="G86" s="1"/>
       <c r="I86" s="2"/>
       <c r="J86" s="2"/>
       <c r="K86" s="2"/>
       <c r="L86" s="1"/>
     </row>
-    <row r="87" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="87" spans="7:12">
       <c r="G87" s="1"/>
       <c r="I87" s="2"/>
       <c r="J87" s="2"/>
       <c r="K87" s="2"/>
       <c r="L87" s="1"/>
     </row>
-    <row r="88" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="88" spans="7:12">
       <c r="G88" s="1"/>
       <c r="I88" s="2"/>
       <c r="J88" s="2"/>
       <c r="K88" s="2"/>
       <c r="L88" s="1"/>
     </row>
-    <row r="89" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="89" spans="7:12">
       <c r="G89" s="1"/>
       <c r="I89" s="2"/>
       <c r="J89" s="2"/>
       <c r="K89" s="2"/>
       <c r="L89" s="1"/>
     </row>
-    <row r="90" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="90" spans="7:12">
       <c r="G90" s="1"/>
       <c r="I90" s="2"/>
       <c r="J90" s="2"/>
       <c r="K90" s="2"/>
       <c r="L90" s="1"/>
     </row>
-    <row r="91" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="91" spans="7:12">
       <c r="G91" s="1"/>
       <c r="I91" s="2"/>
       <c r="J91" s="2"/>
       <c r="K91" s="2"/>
       <c r="L91" s="1"/>
     </row>
-    <row r="92" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="92" spans="7:12">
       <c r="G92" s="1"/>
       <c r="I92" s="2"/>
       <c r="J92" s="2"/>
       <c r="K92" s="2"/>
       <c r="L92" s="1"/>
     </row>
-    <row r="93" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="93" spans="7:12">
       <c r="G93" s="1"/>
       <c r="I93" s="2"/>
       <c r="J93" s="2"/>
       <c r="K93" s="2"/>
       <c r="L93" s="1"/>
     </row>
-    <row r="94" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="94" spans="7:12">
       <c r="G94" s="1"/>
       <c r="I94" s="2"/>
       <c r="J94" s="2"/>
       <c r="K94" s="2"/>
       <c r="L94" s="1"/>
     </row>
-    <row r="95" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="95" spans="7:12">
       <c r="G95" s="1"/>
       <c r="I95" s="2"/>
       <c r="J95" s="2"/>
       <c r="K95" s="2"/>
       <c r="L95" s="1"/>
     </row>
-    <row r="96" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="96" spans="7:12">
       <c r="G96" s="1"/>
       <c r="I96" s="2"/>
       <c r="J96" s="2"/>
       <c r="K96" s="2"/>
       <c r="L96" s="1"/>
     </row>
-    <row r="97" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="97" spans="7:12">
       <c r="G97" s="1"/>
       <c r="I97" s="2"/>
       <c r="J97" s="2"/>
       <c r="K97" s="2"/>
       <c r="L97" s="1"/>
     </row>
-    <row r="98" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="98" spans="7:12">
       <c r="G98" s="1"/>
       <c r="I98" s="2"/>
       <c r="J98" s="2"/>
       <c r="K98" s="2"/>
       <c r="L98" s="1"/>
     </row>
-    <row r="99" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="99" spans="7:12">
       <c r="G99" s="1"/>
       <c r="I99" s="2"/>
       <c r="J99" s="2"/>
       <c r="K99" s="2"/>
       <c r="L99" s="1"/>
     </row>
-    <row r="100" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="100" spans="7:12">
       <c r="G100" s="1"/>
       <c r="I100" s="2"/>
       <c r="J100" s="2"/>
       <c r="K100" s="2"/>
       <c r="L100" s="1"/>
     </row>
-    <row r="101" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="101" spans="7:12">
       <c r="G101" s="1"/>
       <c r="I101" s="2"/>
       <c r="J101" s="2"/>
       <c r="K101" s="2"/>
       <c r="L101" s="1"/>
     </row>
-    <row r="102" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="102" spans="7:12">
       <c r="G102" s="1"/>
       <c r="I102" s="2"/>
       <c r="J102" s="2"/>
       <c r="K102" s="2"/>
       <c r="L102" s="1"/>
     </row>
-    <row r="103" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="103" spans="7:12">
       <c r="G103" s="1"/>
       <c r="I103" s="2"/>
       <c r="J103" s="2"/>
       <c r="K103" s="2"/>
       <c r="L103" s="1"/>
     </row>
-    <row r="104" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="104" spans="7:12">
       <c r="G104" s="1"/>
       <c r="I104" s="2"/>
       <c r="J104" s="2"/>
       <c r="K104" s="2"/>
       <c r="L104" s="1"/>
     </row>
-    <row r="105" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="105" spans="7:12">
       <c r="G105" s="1"/>
       <c r="I105" s="2"/>
       <c r="J105" s="2"/>
       <c r="K105" s="2"/>
       <c r="L105" s="1"/>
     </row>
-    <row r="106" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="106" spans="7:12">
       <c r="G106" s="1"/>
       <c r="I106" s="2"/>
       <c r="J106" s="2"/>
       <c r="K106" s="2"/>
       <c r="L106" s="1"/>
     </row>
-    <row r="107" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="107" spans="7:12">
       <c r="G107" s="1"/>
       <c r="I107" s="2"/>
       <c r="J107" s="2"/>
       <c r="K107" s="2"/>
       <c r="L107" s="1"/>
     </row>
-    <row r="108" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="108" spans="7:12">
       <c r="G108" s="1"/>
       <c r="I108" s="2"/>
       <c r="J108" s="2"/>
       <c r="K108" s="2"/>
       <c r="L108" s="1"/>
     </row>
-    <row r="109" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="109" spans="7:12">
       <c r="G109" s="1"/>
       <c r="I109" s="2"/>
       <c r="J109" s="2"/>
       <c r="K109" s="2"/>
       <c r="L109" s="1"/>
     </row>
-    <row r="110" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="110" spans="7:12">
       <c r="G110" s="1"/>
       <c r="I110" s="2"/>
       <c r="J110" s="2"/>
       <c r="K110" s="2"/>
       <c r="L110" s="1"/>
     </row>
-    <row r="111" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="111" spans="7:12">
       <c r="G111" s="1"/>
       <c r="I111" s="2"/>
       <c r="J111" s="2"/>
       <c r="K111" s="2"/>
       <c r="L111" s="1"/>
     </row>
-    <row r="112" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="112" spans="7:12">
       <c r="G112" s="1"/>
       <c r="I112" s="2"/>
       <c r="J112" s="2"/>
       <c r="K112" s="2"/>
       <c r="L112" s="1"/>
     </row>
-    <row r="113" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="113" spans="7:12">
       <c r="G113" s="1"/>
       <c r="I113" s="2"/>
       <c r="J113" s="2"/>
       <c r="K113" s="2"/>
       <c r="L113" s="1"/>
     </row>
-    <row r="114" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="114" spans="7:12">
       <c r="G114" s="1"/>
       <c r="I114" s="2"/>
       <c r="J114" s="2"/>
       <c r="K114" s="2"/>
       <c r="L114" s="1"/>
     </row>
-    <row r="115" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="115" spans="7:12">
       <c r="G115" s="1"/>
       <c r="I115" s="2"/>
       <c r="J115" s="2"/>
       <c r="K115" s="2"/>
       <c r="L115" s="1"/>
     </row>
-    <row r="116" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="116" spans="7:12">
       <c r="G116" s="1"/>
       <c r="I116" s="2"/>
       <c r="J116" s="2"/>
       <c r="K116" s="2"/>
       <c r="L116" s="1"/>
     </row>
-    <row r="117" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="117" spans="7:12">
       <c r="G117" s="1"/>
       <c r="I117" s="2"/>
       <c r="J117" s="2"/>
       <c r="K117" s="2"/>
       <c r="L117" s="1"/>
     </row>
-    <row r="118" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="118" spans="7:12">
       <c r="G118" s="1"/>
       <c r="I118" s="2"/>
       <c r="J118" s="2"/>
       <c r="K118" s="2"/>
       <c r="L118" s="1"/>
     </row>
-    <row r="119" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="119" spans="7:12">
       <c r="G119" s="1"/>
       <c r="I119" s="2"/>
       <c r="J119" s="2"/>
       <c r="K119" s="2"/>
       <c r="L119" s="1"/>
     </row>
-    <row r="120" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="120" spans="7:12">
       <c r="G120" s="1"/>
       <c r="I120" s="2"/>
       <c r="J120" s="2"/>
       <c r="K120" s="2"/>
       <c r="L120" s="1"/>
     </row>
-    <row r="121" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="121" spans="7:12">
       <c r="G121" s="1"/>
       <c r="I121" s="2"/>
       <c r="J121" s="2"/>
       <c r="K121" s="2"/>
       <c r="L121" s="1"/>
     </row>
-    <row r="122" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="122" spans="7:12">
       <c r="G122" s="1"/>
       <c r="I122" s="2"/>
       <c r="J122" s="2"/>
       <c r="K122" s="2"/>
       <c r="L122" s="1"/>
     </row>
-    <row r="123" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="123" spans="7:12">
       <c r="G123" s="1"/>
       <c r="I123" s="2"/>
       <c r="J123" s="2"/>
       <c r="K123" s="2"/>
       <c r="L123" s="1"/>
     </row>
-    <row r="124" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="124" spans="7:12">
       <c r="G124" s="1"/>
       <c r="I124" s="2"/>
       <c r="J124" s="2"/>
       <c r="K124" s="2"/>
       <c r="L124" s="1"/>
     </row>
-    <row r="125" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="125" spans="7:12">
       <c r="G125" s="1"/>
       <c r="I125" s="2"/>
       <c r="J125" s="2"/>
       <c r="K125" s="2"/>
       <c r="L125" s="1"/>
     </row>
-    <row r="126" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="126" spans="7:12">
       <c r="G126" s="1"/>
       <c r="I126" s="2"/>
       <c r="J126" s="2"/>
       <c r="K126" s="2"/>
       <c r="L126" s="1"/>
     </row>
-    <row r="127" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="127" spans="7:12">
       <c r="G127" s="1"/>
       <c r="I127" s="2"/>
       <c r="J127" s="2"/>
       <c r="K127" s="2"/>
       <c r="L127" s="1"/>
     </row>
-    <row r="128" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="128" spans="7:12">
       <c r="G128" s="1"/>
       <c r="I128" s="2"/>
       <c r="J128" s="2"/>
       <c r="K128" s="2"/>
       <c r="L128" s="1"/>
     </row>
-    <row r="129" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="129" spans="7:12">
       <c r="G129" s="1"/>
       <c r="I129" s="2"/>
       <c r="J129" s="2"/>
       <c r="K129" s="2"/>
       <c r="L129" s="1"/>
     </row>
-    <row r="130" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="130" spans="7:12">
       <c r="G130" s="1"/>
       <c r="I130" s="2"/>
       <c r="J130" s="2"/>
       <c r="K130" s="2"/>
       <c r="L130" s="1"/>
     </row>
-    <row r="131" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="131" spans="7:12">
       <c r="G131" s="1"/>
       <c r="I131" s="2"/>
       <c r="J131" s="2"/>
       <c r="K131" s="2"/>
       <c r="L131" s="1"/>
     </row>
-    <row r="132" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="132" spans="7:12">
       <c r="G132" s="1"/>
       <c r="I132" s="2"/>
       <c r="J132" s="2"/>
       <c r="K132" s="2"/>
       <c r="L132" s="1"/>
     </row>
-    <row r="133" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="133" spans="7:12">
       <c r="G133" s="1"/>
       <c r="I133" s="2"/>
       <c r="J133" s="2"/>
       <c r="K133" s="2"/>
       <c r="L133" s="1"/>
     </row>
-    <row r="134" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="134" spans="7:12">
       <c r="G134" s="1"/>
       <c r="I134" s="2"/>
       <c r="J134" s="2"/>
       <c r="K134" s="2"/>
       <c r="L134" s="1"/>
     </row>
-    <row r="135" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="135" spans="7:12">
       <c r="G135" s="1"/>
       <c r="I135" s="2"/>
       <c r="J135" s="2"/>
       <c r="K135" s="2"/>
       <c r="L135" s="1"/>
     </row>
-    <row r="136" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="136" spans="7:12">
       <c r="G136" s="1"/>
       <c r="I136" s="2"/>
       <c r="J136" s="2"/>
       <c r="K136" s="2"/>
       <c r="L136" s="1"/>
     </row>
-    <row r="137" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="137" spans="7:12">
       <c r="G137" s="1"/>
       <c r="I137" s="2"/>
       <c r="J137" s="2"/>
       <c r="K137" s="2"/>
       <c r="L137" s="1"/>
     </row>
-    <row r="138" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="138" spans="7:12">
       <c r="G138" s="1"/>
       <c r="I138" s="2"/>
       <c r="J138" s="2"/>
       <c r="K138" s="2"/>
       <c r="L138" s="1"/>
     </row>
-    <row r="139" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="139" spans="7:12">
       <c r="G139" s="1"/>
       <c r="I139" s="2"/>
       <c r="J139" s="2"/>
       <c r="K139" s="2"/>
       <c r="L139" s="1"/>
     </row>
-    <row r="140" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="140" spans="7:12">
       <c r="G140" s="1"/>
       <c r="I140" s="2"/>
       <c r="J140" s="2"/>
       <c r="K140" s="2"/>
       <c r="L140" s="1"/>
     </row>
-    <row r="141" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="141" spans="7:12">
       <c r="G141" s="1"/>
       <c r="I141" s="2"/>
       <c r="J141" s="2"/>
       <c r="K141" s="2"/>
       <c r="L141" s="1"/>
     </row>
-    <row r="142" spans="7:12" x14ac:dyDescent="0.3">
+    <row r="142" spans="7:12">
       <c r="G142" s="1"/>
       <c r="I142" s="2"/>
       <c r="J142" s="2"/>
       <c r="K142" s="2"/>
       <c r="L142" s="1"/>
     </row>
-    <row r="143" spans="7:12" x14ac:dyDescent="0.3">
-      <c r="G143" s="1"/>
-      <c r="I143" s="2"/>
-      <c r="J143" s="2"/>
-      <c r="K143" s="2"/>
-      <c r="L143" s="1"/>
-    </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="S2:X2"/>
-    <mergeCell ref="A1:Q1"/>
+  <mergeCells count="1">
+    <mergeCell ref="S1:X1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
completed the compare sql result gherkin step
</commit_message>
<xml_diff>
--- a/src/test.dataExchange/resources/filesToIngest/mfpDemo.xlsx
+++ b/src/test.dataExchange/resources/filesToIngest/mfpDemo.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rachowdhury\Documents\Software\mtf-dm-automation-test-api\src\test.dataExchange\resources\filesToIngest\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mthomas\Documents\mtf-dm-automation-test-api\src\test.dataExchange\resources\filesToIngest\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36BE23CA-5E5E-4851-8244-4EF155EC55F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05182816-238F-438C-AD6F-38ECAFB78DDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{19ED86A4-C2F1-4297-8EB6-669432289AF5}"/>
+    <workbookView xWindow="20070" yWindow="-2880" windowWidth="21730" windowHeight="11570" xr2:uid="{19ED86A4-C2F1-4297-8EB6-669432289AF5}"/>
   </bookViews>
   <sheets>
     <sheet name="MFP Pricing File - Data" sheetId="1" r:id="rId1"/>
@@ -111,7 +111,7 @@
   <numFmts count="1">
     <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -983,16 +983,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9669907-CFD9-41C9-BD8E-B33EA6BCF659}">
   <dimension ref="A1:X142"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="4" max="4" width="12.3984375" customWidth="1"/>
-    <col min="7" max="7" width="16.8984375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.296875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.3984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.44140625" customWidth="1"/>
+    <col min="7" max="7" width="16.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" s="3" customFormat="1" ht="90.75" customHeight="1">
+    <row r="1" spans="1:24" s="3" customFormat="1" ht="90.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1042,7 +1042,7 @@
       <c r="W1" s="5"/>
       <c r="X1" s="5"/>
     </row>
-    <row r="2" spans="1:24">
+    <row r="2" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2026</v>
       </c>
@@ -1080,7 +1080,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:24">
+    <row r="3" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2026</v>
       </c>
@@ -1118,7 +1118,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:24">
+    <row r="4" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2026</v>
       </c>
@@ -1156,966 +1156,966 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:24">
+    <row r="5" spans="1:24" x14ac:dyDescent="0.3">
       <c r="G5" s="1"/>
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
       <c r="L5" s="1"/>
     </row>
-    <row r="6" spans="1:24">
+    <row r="6" spans="1:24" x14ac:dyDescent="0.3">
       <c r="G6" s="1"/>
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
       <c r="K6" s="2"/>
       <c r="L6" s="1"/>
     </row>
-    <row r="7" spans="1:24">
+    <row r="7" spans="1:24" x14ac:dyDescent="0.3">
       <c r="G7" s="1"/>
       <c r="I7" s="2"/>
       <c r="J7" s="2"/>
       <c r="K7" s="2"/>
       <c r="L7" s="1"/>
     </row>
-    <row r="8" spans="1:24">
+    <row r="8" spans="1:24" x14ac:dyDescent="0.3">
       <c r="G8" s="1"/>
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
       <c r="K8" s="2"/>
       <c r="L8" s="1"/>
     </row>
-    <row r="9" spans="1:24">
+    <row r="9" spans="1:24" x14ac:dyDescent="0.3">
       <c r="G9" s="1"/>
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
       <c r="K9" s="2"/>
       <c r="L9" s="1"/>
     </row>
-    <row r="10" spans="1:24">
+    <row r="10" spans="1:24" x14ac:dyDescent="0.3">
       <c r="G10" s="1"/>
       <c r="I10" s="2"/>
       <c r="J10" s="2"/>
       <c r="K10" s="2"/>
       <c r="L10" s="1"/>
     </row>
-    <row r="11" spans="1:24">
+    <row r="11" spans="1:24" x14ac:dyDescent="0.3">
       <c r="G11" s="1"/>
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
       <c r="K11" s="2"/>
       <c r="L11" s="1"/>
     </row>
-    <row r="12" spans="1:24">
+    <row r="12" spans="1:24" x14ac:dyDescent="0.3">
       <c r="G12" s="1"/>
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
       <c r="L12" s="1"/>
     </row>
-    <row r="13" spans="1:24">
+    <row r="13" spans="1:24" x14ac:dyDescent="0.3">
       <c r="G13" s="1"/>
       <c r="I13" s="2"/>
       <c r="J13" s="2"/>
       <c r="K13" s="2"/>
       <c r="L13" s="1"/>
     </row>
-    <row r="14" spans="1:24">
+    <row r="14" spans="1:24" x14ac:dyDescent="0.3">
       <c r="G14" s="1"/>
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>
       <c r="L14" s="1"/>
     </row>
-    <row r="15" spans="1:24">
+    <row r="15" spans="1:24" x14ac:dyDescent="0.3">
       <c r="G15" s="1"/>
       <c r="I15" s="2"/>
       <c r="J15" s="2"/>
       <c r="K15" s="2"/>
       <c r="L15" s="1"/>
     </row>
-    <row r="16" spans="1:24">
+    <row r="16" spans="1:24" x14ac:dyDescent="0.3">
       <c r="G16" s="1"/>
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
       <c r="K16" s="2"/>
       <c r="L16" s="1"/>
     </row>
-    <row r="17" spans="7:12">
+    <row r="17" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G17" s="1"/>
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
       <c r="K17" s="2"/>
       <c r="L17" s="1"/>
     </row>
-    <row r="18" spans="7:12">
+    <row r="18" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G18" s="1"/>
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
       <c r="K18" s="2"/>
       <c r="L18" s="1"/>
     </row>
-    <row r="19" spans="7:12">
+    <row r="19" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G19" s="1"/>
       <c r="I19" s="2"/>
       <c r="J19" s="2"/>
       <c r="K19" s="2"/>
       <c r="L19" s="1"/>
     </row>
-    <row r="20" spans="7:12">
+    <row r="20" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G20" s="1"/>
       <c r="I20" s="2"/>
       <c r="J20" s="2"/>
       <c r="K20" s="2"/>
       <c r="L20" s="1"/>
     </row>
-    <row r="21" spans="7:12">
+    <row r="21" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G21" s="1"/>
       <c r="I21" s="2"/>
       <c r="J21" s="2"/>
       <c r="K21" s="2"/>
       <c r="L21" s="1"/>
     </row>
-    <row r="22" spans="7:12">
+    <row r="22" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G22" s="1"/>
       <c r="I22" s="2"/>
       <c r="J22" s="2"/>
       <c r="K22" s="2"/>
       <c r="L22" s="1"/>
     </row>
-    <row r="23" spans="7:12">
+    <row r="23" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G23" s="1"/>
       <c r="I23" s="2"/>
       <c r="J23" s="2"/>
       <c r="K23" s="2"/>
       <c r="L23" s="1"/>
     </row>
-    <row r="24" spans="7:12">
+    <row r="24" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G24" s="1"/>
       <c r="I24" s="2"/>
       <c r="J24" s="2"/>
       <c r="K24" s="2"/>
       <c r="L24" s="1"/>
     </row>
-    <row r="25" spans="7:12">
+    <row r="25" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G25" s="1"/>
       <c r="I25" s="2"/>
       <c r="J25" s="2"/>
       <c r="K25" s="2"/>
       <c r="L25" s="1"/>
     </row>
-    <row r="26" spans="7:12">
+    <row r="26" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G26" s="1"/>
       <c r="I26" s="2"/>
       <c r="J26" s="2"/>
       <c r="K26" s="2"/>
       <c r="L26" s="1"/>
     </row>
-    <row r="27" spans="7:12">
+    <row r="27" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G27" s="1"/>
       <c r="I27" s="2"/>
       <c r="J27" s="2"/>
       <c r="K27" s="2"/>
       <c r="L27" s="1"/>
     </row>
-    <row r="28" spans="7:12">
+    <row r="28" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G28" s="1"/>
       <c r="I28" s="2"/>
       <c r="J28" s="2"/>
       <c r="K28" s="2"/>
       <c r="L28" s="1"/>
     </row>
-    <row r="29" spans="7:12">
+    <row r="29" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G29" s="1"/>
       <c r="I29" s="2"/>
       <c r="J29" s="2"/>
       <c r="K29" s="2"/>
       <c r="L29" s="1"/>
     </row>
-    <row r="30" spans="7:12">
+    <row r="30" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G30" s="1"/>
       <c r="I30" s="2"/>
       <c r="J30" s="2"/>
       <c r="K30" s="2"/>
       <c r="L30" s="1"/>
     </row>
-    <row r="31" spans="7:12">
+    <row r="31" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G31" s="1"/>
       <c r="I31" s="2"/>
       <c r="J31" s="2"/>
       <c r="K31" s="2"/>
       <c r="L31" s="1"/>
     </row>
-    <row r="32" spans="7:12">
+    <row r="32" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G32" s="1"/>
       <c r="I32" s="2"/>
       <c r="J32" s="2"/>
       <c r="K32" s="2"/>
       <c r="L32" s="1"/>
     </row>
-    <row r="33" spans="7:12">
+    <row r="33" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G33" s="1"/>
       <c r="I33" s="2"/>
       <c r="J33" s="2"/>
       <c r="K33" s="2"/>
       <c r="L33" s="1"/>
     </row>
-    <row r="34" spans="7:12">
+    <row r="34" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G34" s="1"/>
       <c r="I34" s="2"/>
       <c r="J34" s="2"/>
       <c r="K34" s="2"/>
       <c r="L34" s="1"/>
     </row>
-    <row r="35" spans="7:12">
+    <row r="35" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G35" s="1"/>
       <c r="I35" s="2"/>
       <c r="J35" s="2"/>
       <c r="K35" s="2"/>
       <c r="L35" s="1"/>
     </row>
-    <row r="36" spans="7:12">
+    <row r="36" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G36" s="1"/>
       <c r="I36" s="2"/>
       <c r="J36" s="2"/>
       <c r="K36" s="2"/>
       <c r="L36" s="1"/>
     </row>
-    <row r="37" spans="7:12">
+    <row r="37" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G37" s="1"/>
       <c r="I37" s="2"/>
       <c r="J37" s="2"/>
       <c r="K37" s="2"/>
       <c r="L37" s="1"/>
     </row>
-    <row r="38" spans="7:12">
+    <row r="38" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G38" s="1"/>
       <c r="I38" s="2"/>
       <c r="J38" s="2"/>
       <c r="K38" s="2"/>
       <c r="L38" s="1"/>
     </row>
-    <row r="39" spans="7:12">
+    <row r="39" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G39" s="1"/>
       <c r="I39" s="2"/>
       <c r="J39" s="2"/>
       <c r="K39" s="2"/>
       <c r="L39" s="1"/>
     </row>
-    <row r="40" spans="7:12">
+    <row r="40" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G40" s="1"/>
       <c r="I40" s="2"/>
       <c r="J40" s="2"/>
       <c r="K40" s="2"/>
       <c r="L40" s="1"/>
     </row>
-    <row r="41" spans="7:12">
+    <row r="41" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G41" s="1"/>
       <c r="I41" s="2"/>
       <c r="J41" s="2"/>
       <c r="K41" s="2"/>
       <c r="L41" s="1"/>
     </row>
-    <row r="42" spans="7:12">
+    <row r="42" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G42" s="1"/>
       <c r="I42" s="2"/>
       <c r="J42" s="2"/>
       <c r="K42" s="2"/>
       <c r="L42" s="1"/>
     </row>
-    <row r="43" spans="7:12">
+    <row r="43" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G43" s="1"/>
       <c r="I43" s="2"/>
       <c r="J43" s="2"/>
       <c r="K43" s="2"/>
       <c r="L43" s="1"/>
     </row>
-    <row r="44" spans="7:12">
+    <row r="44" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G44" s="1"/>
       <c r="I44" s="2"/>
       <c r="J44" s="2"/>
       <c r="K44" s="2"/>
       <c r="L44" s="1"/>
     </row>
-    <row r="45" spans="7:12">
+    <row r="45" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G45" s="1"/>
       <c r="I45" s="2"/>
       <c r="J45" s="2"/>
       <c r="K45" s="2"/>
       <c r="L45" s="1"/>
     </row>
-    <row r="46" spans="7:12">
+    <row r="46" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G46" s="1"/>
       <c r="I46" s="2"/>
       <c r="J46" s="2"/>
       <c r="K46" s="2"/>
       <c r="L46" s="1"/>
     </row>
-    <row r="47" spans="7:12">
+    <row r="47" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G47" s="1"/>
       <c r="I47" s="2"/>
       <c r="J47" s="2"/>
       <c r="K47" s="2"/>
       <c r="L47" s="1"/>
     </row>
-    <row r="48" spans="7:12">
+    <row r="48" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G48" s="1"/>
       <c r="I48" s="2"/>
       <c r="J48" s="2"/>
       <c r="K48" s="2"/>
       <c r="L48" s="1"/>
     </row>
-    <row r="49" spans="7:12">
+    <row r="49" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G49" s="1"/>
       <c r="I49" s="2"/>
       <c r="J49" s="2"/>
       <c r="K49" s="2"/>
       <c r="L49" s="1"/>
     </row>
-    <row r="50" spans="7:12">
+    <row r="50" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G50" s="1"/>
       <c r="I50" s="2"/>
       <c r="J50" s="2"/>
       <c r="K50" s="2"/>
       <c r="L50" s="1"/>
     </row>
-    <row r="51" spans="7:12">
+    <row r="51" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G51" s="1"/>
       <c r="I51" s="2"/>
       <c r="J51" s="2"/>
       <c r="K51" s="2"/>
       <c r="L51" s="1"/>
     </row>
-    <row r="52" spans="7:12">
+    <row r="52" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G52" s="1"/>
       <c r="I52" s="2"/>
       <c r="J52" s="2"/>
       <c r="K52" s="2"/>
       <c r="L52" s="1"/>
     </row>
-    <row r="53" spans="7:12">
+    <row r="53" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G53" s="1"/>
       <c r="I53" s="2"/>
       <c r="J53" s="2"/>
       <c r="K53" s="2"/>
       <c r="L53" s="1"/>
     </row>
-    <row r="54" spans="7:12">
+    <row r="54" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G54" s="1"/>
       <c r="I54" s="2"/>
       <c r="J54" s="2"/>
       <c r="K54" s="2"/>
       <c r="L54" s="1"/>
     </row>
-    <row r="55" spans="7:12">
+    <row r="55" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G55" s="1"/>
       <c r="I55" s="2"/>
       <c r="J55" s="2"/>
       <c r="K55" s="2"/>
       <c r="L55" s="1"/>
     </row>
-    <row r="56" spans="7:12">
+    <row r="56" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G56" s="1"/>
       <c r="I56" s="2"/>
       <c r="J56" s="2"/>
       <c r="K56" s="2"/>
       <c r="L56" s="1"/>
     </row>
-    <row r="57" spans="7:12">
+    <row r="57" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G57" s="1"/>
       <c r="I57" s="2"/>
       <c r="J57" s="2"/>
       <c r="K57" s="2"/>
       <c r="L57" s="1"/>
     </row>
-    <row r="58" spans="7:12">
+    <row r="58" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G58" s="1"/>
       <c r="I58" s="2"/>
       <c r="J58" s="2"/>
       <c r="K58" s="2"/>
       <c r="L58" s="1"/>
     </row>
-    <row r="59" spans="7:12">
+    <row r="59" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G59" s="1"/>
       <c r="I59" s="2"/>
       <c r="J59" s="2"/>
       <c r="K59" s="2"/>
       <c r="L59" s="1"/>
     </row>
-    <row r="60" spans="7:12">
+    <row r="60" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G60" s="1"/>
       <c r="I60" s="2"/>
       <c r="J60" s="2"/>
       <c r="K60" s="2"/>
       <c r="L60" s="1"/>
     </row>
-    <row r="61" spans="7:12">
+    <row r="61" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G61" s="1"/>
       <c r="I61" s="2"/>
       <c r="J61" s="2"/>
       <c r="K61" s="2"/>
       <c r="L61" s="1"/>
     </row>
-    <row r="62" spans="7:12">
+    <row r="62" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G62" s="1"/>
       <c r="I62" s="2"/>
       <c r="J62" s="2"/>
       <c r="K62" s="2"/>
       <c r="L62" s="1"/>
     </row>
-    <row r="63" spans="7:12">
+    <row r="63" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G63" s="1"/>
       <c r="I63" s="2"/>
       <c r="J63" s="2"/>
       <c r="K63" s="2"/>
       <c r="L63" s="1"/>
     </row>
-    <row r="64" spans="7:12">
+    <row r="64" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G64" s="1"/>
       <c r="I64" s="2"/>
       <c r="J64" s="2"/>
       <c r="K64" s="2"/>
       <c r="L64" s="1"/>
     </row>
-    <row r="65" spans="7:12">
+    <row r="65" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G65" s="1"/>
       <c r="I65" s="2"/>
       <c r="J65" s="2"/>
       <c r="K65" s="2"/>
       <c r="L65" s="1"/>
     </row>
-    <row r="66" spans="7:12">
+    <row r="66" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G66" s="1"/>
       <c r="I66" s="2"/>
       <c r="J66" s="2"/>
       <c r="K66" s="2"/>
       <c r="L66" s="1"/>
     </row>
-    <row r="67" spans="7:12">
+    <row r="67" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G67" s="1"/>
       <c r="I67" s="2"/>
       <c r="J67" s="2"/>
       <c r="K67" s="2"/>
       <c r="L67" s="1"/>
     </row>
-    <row r="68" spans="7:12">
+    <row r="68" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G68" s="1"/>
       <c r="I68" s="2"/>
       <c r="J68" s="2"/>
       <c r="K68" s="2"/>
       <c r="L68" s="1"/>
     </row>
-    <row r="69" spans="7:12">
+    <row r="69" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G69" s="1"/>
       <c r="I69" s="2"/>
       <c r="J69" s="2"/>
       <c r="K69" s="2"/>
       <c r="L69" s="1"/>
     </row>
-    <row r="70" spans="7:12">
+    <row r="70" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G70" s="1"/>
       <c r="I70" s="2"/>
       <c r="J70" s="2"/>
       <c r="K70" s="2"/>
       <c r="L70" s="1"/>
     </row>
-    <row r="71" spans="7:12">
+    <row r="71" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G71" s="1"/>
       <c r="I71" s="2"/>
       <c r="J71" s="2"/>
       <c r="K71" s="2"/>
       <c r="L71" s="1"/>
     </row>
-    <row r="72" spans="7:12">
+    <row r="72" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G72" s="1"/>
       <c r="I72" s="2"/>
       <c r="J72" s="2"/>
       <c r="K72" s="2"/>
       <c r="L72" s="1"/>
     </row>
-    <row r="73" spans="7:12">
+    <row r="73" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G73" s="1"/>
       <c r="I73" s="2"/>
       <c r="J73" s="2"/>
       <c r="K73" s="2"/>
       <c r="L73" s="1"/>
     </row>
-    <row r="74" spans="7:12">
+    <row r="74" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G74" s="1"/>
       <c r="I74" s="2"/>
       <c r="J74" s="2"/>
       <c r="K74" s="2"/>
       <c r="L74" s="1"/>
     </row>
-    <row r="75" spans="7:12">
+    <row r="75" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G75" s="1"/>
       <c r="I75" s="2"/>
       <c r="J75" s="2"/>
       <c r="K75" s="2"/>
       <c r="L75" s="1"/>
     </row>
-    <row r="76" spans="7:12">
+    <row r="76" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G76" s="1"/>
       <c r="I76" s="2"/>
       <c r="J76" s="2"/>
       <c r="K76" s="2"/>
       <c r="L76" s="1"/>
     </row>
-    <row r="77" spans="7:12">
+    <row r="77" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G77" s="1"/>
       <c r="I77" s="2"/>
       <c r="J77" s="2"/>
       <c r="K77" s="2"/>
       <c r="L77" s="1"/>
     </row>
-    <row r="78" spans="7:12">
+    <row r="78" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G78" s="1"/>
       <c r="I78" s="2"/>
       <c r="J78" s="2"/>
       <c r="K78" s="2"/>
       <c r="L78" s="1"/>
     </row>
-    <row r="79" spans="7:12">
+    <row r="79" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G79" s="1"/>
       <c r="I79" s="2"/>
       <c r="J79" s="2"/>
       <c r="K79" s="2"/>
       <c r="L79" s="1"/>
     </row>
-    <row r="80" spans="7:12">
+    <row r="80" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G80" s="1"/>
       <c r="I80" s="2"/>
       <c r="J80" s="2"/>
       <c r="K80" s="2"/>
       <c r="L80" s="1"/>
     </row>
-    <row r="81" spans="7:12">
+    <row r="81" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G81" s="1"/>
       <c r="I81" s="2"/>
       <c r="J81" s="2"/>
       <c r="K81" s="2"/>
       <c r="L81" s="1"/>
     </row>
-    <row r="82" spans="7:12">
+    <row r="82" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G82" s="1"/>
       <c r="I82" s="2"/>
       <c r="J82" s="2"/>
       <c r="K82" s="2"/>
       <c r="L82" s="1"/>
     </row>
-    <row r="83" spans="7:12">
+    <row r="83" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G83" s="1"/>
       <c r="I83" s="2"/>
       <c r="J83" s="2"/>
       <c r="K83" s="2"/>
       <c r="L83" s="1"/>
     </row>
-    <row r="84" spans="7:12">
+    <row r="84" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G84" s="1"/>
       <c r="I84" s="2"/>
       <c r="J84" s="2"/>
       <c r="K84" s="2"/>
       <c r="L84" s="1"/>
     </row>
-    <row r="85" spans="7:12">
+    <row r="85" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G85" s="1"/>
       <c r="I85" s="2"/>
       <c r="J85" s="2"/>
       <c r="K85" s="2"/>
       <c r="L85" s="1"/>
     </row>
-    <row r="86" spans="7:12">
+    <row r="86" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G86" s="1"/>
       <c r="I86" s="2"/>
       <c r="J86" s="2"/>
       <c r="K86" s="2"/>
       <c r="L86" s="1"/>
     </row>
-    <row r="87" spans="7:12">
+    <row r="87" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G87" s="1"/>
       <c r="I87" s="2"/>
       <c r="J87" s="2"/>
       <c r="K87" s="2"/>
       <c r="L87" s="1"/>
     </row>
-    <row r="88" spans="7:12">
+    <row r="88" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G88" s="1"/>
       <c r="I88" s="2"/>
       <c r="J88" s="2"/>
       <c r="K88" s="2"/>
       <c r="L88" s="1"/>
     </row>
-    <row r="89" spans="7:12">
+    <row r="89" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G89" s="1"/>
       <c r="I89" s="2"/>
       <c r="J89" s="2"/>
       <c r="K89" s="2"/>
       <c r="L89" s="1"/>
     </row>
-    <row r="90" spans="7:12">
+    <row r="90" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G90" s="1"/>
       <c r="I90" s="2"/>
       <c r="J90" s="2"/>
       <c r="K90" s="2"/>
       <c r="L90" s="1"/>
     </row>
-    <row r="91" spans="7:12">
+    <row r="91" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G91" s="1"/>
       <c r="I91" s="2"/>
       <c r="J91" s="2"/>
       <c r="K91" s="2"/>
       <c r="L91" s="1"/>
     </row>
-    <row r="92" spans="7:12">
+    <row r="92" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G92" s="1"/>
       <c r="I92" s="2"/>
       <c r="J92" s="2"/>
       <c r="K92" s="2"/>
       <c r="L92" s="1"/>
     </row>
-    <row r="93" spans="7:12">
+    <row r="93" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G93" s="1"/>
       <c r="I93" s="2"/>
       <c r="J93" s="2"/>
       <c r="K93" s="2"/>
       <c r="L93" s="1"/>
     </row>
-    <row r="94" spans="7:12">
+    <row r="94" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G94" s="1"/>
       <c r="I94" s="2"/>
       <c r="J94" s="2"/>
       <c r="K94" s="2"/>
       <c r="L94" s="1"/>
     </row>
-    <row r="95" spans="7:12">
+    <row r="95" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G95" s="1"/>
       <c r="I95" s="2"/>
       <c r="J95" s="2"/>
       <c r="K95" s="2"/>
       <c r="L95" s="1"/>
     </row>
-    <row r="96" spans="7:12">
+    <row r="96" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G96" s="1"/>
       <c r="I96" s="2"/>
       <c r="J96" s="2"/>
       <c r="K96" s="2"/>
       <c r="L96" s="1"/>
     </row>
-    <row r="97" spans="7:12">
+    <row r="97" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G97" s="1"/>
       <c r="I97" s="2"/>
       <c r="J97" s="2"/>
       <c r="K97" s="2"/>
       <c r="L97" s="1"/>
     </row>
-    <row r="98" spans="7:12">
+    <row r="98" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G98" s="1"/>
       <c r="I98" s="2"/>
       <c r="J98" s="2"/>
       <c r="K98" s="2"/>
       <c r="L98" s="1"/>
     </row>
-    <row r="99" spans="7:12">
+    <row r="99" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G99" s="1"/>
       <c r="I99" s="2"/>
       <c r="J99" s="2"/>
       <c r="K99" s="2"/>
       <c r="L99" s="1"/>
     </row>
-    <row r="100" spans="7:12">
+    <row r="100" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G100" s="1"/>
       <c r="I100" s="2"/>
       <c r="J100" s="2"/>
       <c r="K100" s="2"/>
       <c r="L100" s="1"/>
     </row>
-    <row r="101" spans="7:12">
+    <row r="101" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G101" s="1"/>
       <c r="I101" s="2"/>
       <c r="J101" s="2"/>
       <c r="K101" s="2"/>
       <c r="L101" s="1"/>
     </row>
-    <row r="102" spans="7:12">
+    <row r="102" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G102" s="1"/>
       <c r="I102" s="2"/>
       <c r="J102" s="2"/>
       <c r="K102" s="2"/>
       <c r="L102" s="1"/>
     </row>
-    <row r="103" spans="7:12">
+    <row r="103" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G103" s="1"/>
       <c r="I103" s="2"/>
       <c r="J103" s="2"/>
       <c r="K103" s="2"/>
       <c r="L103" s="1"/>
     </row>
-    <row r="104" spans="7:12">
+    <row r="104" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G104" s="1"/>
       <c r="I104" s="2"/>
       <c r="J104" s="2"/>
       <c r="K104" s="2"/>
       <c r="L104" s="1"/>
     </row>
-    <row r="105" spans="7:12">
+    <row r="105" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G105" s="1"/>
       <c r="I105" s="2"/>
       <c r="J105" s="2"/>
       <c r="K105" s="2"/>
       <c r="L105" s="1"/>
     </row>
-    <row r="106" spans="7:12">
+    <row r="106" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G106" s="1"/>
       <c r="I106" s="2"/>
       <c r="J106" s="2"/>
       <c r="K106" s="2"/>
       <c r="L106" s="1"/>
     </row>
-    <row r="107" spans="7:12">
+    <row r="107" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G107" s="1"/>
       <c r="I107" s="2"/>
       <c r="J107" s="2"/>
       <c r="K107" s="2"/>
       <c r="L107" s="1"/>
     </row>
-    <row r="108" spans="7:12">
+    <row r="108" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G108" s="1"/>
       <c r="I108" s="2"/>
       <c r="J108" s="2"/>
       <c r="K108" s="2"/>
       <c r="L108" s="1"/>
     </row>
-    <row r="109" spans="7:12">
+    <row r="109" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G109" s="1"/>
       <c r="I109" s="2"/>
       <c r="J109" s="2"/>
       <c r="K109" s="2"/>
       <c r="L109" s="1"/>
     </row>
-    <row r="110" spans="7:12">
+    <row r="110" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G110" s="1"/>
       <c r="I110" s="2"/>
       <c r="J110" s="2"/>
       <c r="K110" s="2"/>
       <c r="L110" s="1"/>
     </row>
-    <row r="111" spans="7:12">
+    <row r="111" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G111" s="1"/>
       <c r="I111" s="2"/>
       <c r="J111" s="2"/>
       <c r="K111" s="2"/>
       <c r="L111" s="1"/>
     </row>
-    <row r="112" spans="7:12">
+    <row r="112" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G112" s="1"/>
       <c r="I112" s="2"/>
       <c r="J112" s="2"/>
       <c r="K112" s="2"/>
       <c r="L112" s="1"/>
     </row>
-    <row r="113" spans="7:12">
+    <row r="113" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G113" s="1"/>
       <c r="I113" s="2"/>
       <c r="J113" s="2"/>
       <c r="K113" s="2"/>
       <c r="L113" s="1"/>
     </row>
-    <row r="114" spans="7:12">
+    <row r="114" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G114" s="1"/>
       <c r="I114" s="2"/>
       <c r="J114" s="2"/>
       <c r="K114" s="2"/>
       <c r="L114" s="1"/>
     </row>
-    <row r="115" spans="7:12">
+    <row r="115" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G115" s="1"/>
       <c r="I115" s="2"/>
       <c r="J115" s="2"/>
       <c r="K115" s="2"/>
       <c r="L115" s="1"/>
     </row>
-    <row r="116" spans="7:12">
+    <row r="116" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G116" s="1"/>
       <c r="I116" s="2"/>
       <c r="J116" s="2"/>
       <c r="K116" s="2"/>
       <c r="L116" s="1"/>
     </row>
-    <row r="117" spans="7:12">
+    <row r="117" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G117" s="1"/>
       <c r="I117" s="2"/>
       <c r="J117" s="2"/>
       <c r="K117" s="2"/>
       <c r="L117" s="1"/>
     </row>
-    <row r="118" spans="7:12">
+    <row r="118" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G118" s="1"/>
       <c r="I118" s="2"/>
       <c r="J118" s="2"/>
       <c r="K118" s="2"/>
       <c r="L118" s="1"/>
     </row>
-    <row r="119" spans="7:12">
+    <row r="119" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G119" s="1"/>
       <c r="I119" s="2"/>
       <c r="J119" s="2"/>
       <c r="K119" s="2"/>
       <c r="L119" s="1"/>
     </row>
-    <row r="120" spans="7:12">
+    <row r="120" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G120" s="1"/>
       <c r="I120" s="2"/>
       <c r="J120" s="2"/>
       <c r="K120" s="2"/>
       <c r="L120" s="1"/>
     </row>
-    <row r="121" spans="7:12">
+    <row r="121" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G121" s="1"/>
       <c r="I121" s="2"/>
       <c r="J121" s="2"/>
       <c r="K121" s="2"/>
       <c r="L121" s="1"/>
     </row>
-    <row r="122" spans="7:12">
+    <row r="122" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G122" s="1"/>
       <c r="I122" s="2"/>
       <c r="J122" s="2"/>
       <c r="K122" s="2"/>
       <c r="L122" s="1"/>
     </row>
-    <row r="123" spans="7:12">
+    <row r="123" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G123" s="1"/>
       <c r="I123" s="2"/>
       <c r="J123" s="2"/>
       <c r="K123" s="2"/>
       <c r="L123" s="1"/>
     </row>
-    <row r="124" spans="7:12">
+    <row r="124" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G124" s="1"/>
       <c r="I124" s="2"/>
       <c r="J124" s="2"/>
       <c r="K124" s="2"/>
       <c r="L124" s="1"/>
     </row>
-    <row r="125" spans="7:12">
+    <row r="125" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G125" s="1"/>
       <c r="I125" s="2"/>
       <c r="J125" s="2"/>
       <c r="K125" s="2"/>
       <c r="L125" s="1"/>
     </row>
-    <row r="126" spans="7:12">
+    <row r="126" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G126" s="1"/>
       <c r="I126" s="2"/>
       <c r="J126" s="2"/>
       <c r="K126" s="2"/>
       <c r="L126" s="1"/>
     </row>
-    <row r="127" spans="7:12">
+    <row r="127" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G127" s="1"/>
       <c r="I127" s="2"/>
       <c r="J127" s="2"/>
       <c r="K127" s="2"/>
       <c r="L127" s="1"/>
     </row>
-    <row r="128" spans="7:12">
+    <row r="128" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G128" s="1"/>
       <c r="I128" s="2"/>
       <c r="J128" s="2"/>
       <c r="K128" s="2"/>
       <c r="L128" s="1"/>
     </row>
-    <row r="129" spans="7:12">
+    <row r="129" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G129" s="1"/>
       <c r="I129" s="2"/>
       <c r="J129" s="2"/>
       <c r="K129" s="2"/>
       <c r="L129" s="1"/>
     </row>
-    <row r="130" spans="7:12">
+    <row r="130" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G130" s="1"/>
       <c r="I130" s="2"/>
       <c r="J130" s="2"/>
       <c r="K130" s="2"/>
       <c r="L130" s="1"/>
     </row>
-    <row r="131" spans="7:12">
+    <row r="131" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G131" s="1"/>
       <c r="I131" s="2"/>
       <c r="J131" s="2"/>
       <c r="K131" s="2"/>
       <c r="L131" s="1"/>
     </row>
-    <row r="132" spans="7:12">
+    <row r="132" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G132" s="1"/>
       <c r="I132" s="2"/>
       <c r="J132" s="2"/>
       <c r="K132" s="2"/>
       <c r="L132" s="1"/>
     </row>
-    <row r="133" spans="7:12">
+    <row r="133" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G133" s="1"/>
       <c r="I133" s="2"/>
       <c r="J133" s="2"/>
       <c r="K133" s="2"/>
       <c r="L133" s="1"/>
     </row>
-    <row r="134" spans="7:12">
+    <row r="134" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G134" s="1"/>
       <c r="I134" s="2"/>
       <c r="J134" s="2"/>
       <c r="K134" s="2"/>
       <c r="L134" s="1"/>
     </row>
-    <row r="135" spans="7:12">
+    <row r="135" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G135" s="1"/>
       <c r="I135" s="2"/>
       <c r="J135" s="2"/>
       <c r="K135" s="2"/>
       <c r="L135" s="1"/>
     </row>
-    <row r="136" spans="7:12">
+    <row r="136" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G136" s="1"/>
       <c r="I136" s="2"/>
       <c r="J136" s="2"/>
       <c r="K136" s="2"/>
       <c r="L136" s="1"/>
     </row>
-    <row r="137" spans="7:12">
+    <row r="137" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G137" s="1"/>
       <c r="I137" s="2"/>
       <c r="J137" s="2"/>
       <c r="K137" s="2"/>
       <c r="L137" s="1"/>
     </row>
-    <row r="138" spans="7:12">
+    <row r="138" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G138" s="1"/>
       <c r="I138" s="2"/>
       <c r="J138" s="2"/>
       <c r="K138" s="2"/>
       <c r="L138" s="1"/>
     </row>
-    <row r="139" spans="7:12">
+    <row r="139" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G139" s="1"/>
       <c r="I139" s="2"/>
       <c r="J139" s="2"/>
       <c r="K139" s="2"/>
       <c r="L139" s="1"/>
     </row>
-    <row r="140" spans="7:12">
+    <row r="140" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G140" s="1"/>
       <c r="I140" s="2"/>
       <c r="J140" s="2"/>
       <c r="K140" s="2"/>
       <c r="L140" s="1"/>
     </row>
-    <row r="141" spans="7:12">
+    <row r="141" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G141" s="1"/>
       <c r="I141" s="2"/>
       <c r="J141" s="2"/>
       <c r="K141" s="2"/>
       <c r="L141" s="1"/>
     </row>
-    <row r="142" spans="7:12">
+    <row r="142" spans="7:12" x14ac:dyDescent="0.3">
       <c r="G142" s="1"/>
       <c r="I142" s="2"/>
       <c r="J142" s="2"/>

</xml_diff>